<commit_message>
PT: modo stand Web Summit (/stand, guia de 3 min, recomeçar e reinício automático), Assistente offline na página real, respostas demo revistas, nota sísmica formatada com zonas de Lisboa; limpeza do francês nos PDF (MEP, processo BET), título «Nova conversa», IVA reduzido PT na declaração; SW v10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015pifK7S6HJbKkARLCtXv6a
</commit_message>
<xml_diff>
--- a/frontend/public/demo-assets/Orcamento_Moradia_Martins.xlsx
+++ b/frontend/public/demo-assets/Orcamento_Moradia_Martins.xlsx
@@ -36,7 +36,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000E4D4A"/>
+      <color rgb="00203B2D"/>
       <sz val="14"/>
     </font>
     <font>
@@ -74,12 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000E4D4A"/>
+        <fgColor rgb="00203B2D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7EDED"/>
+        <fgColor rgb="00E9EBEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Madres de lamelado colado GL24h 115 × 360 (×5)</t>
+          <t>Madres de lamelado colado GL24h 100 × 240 (×5)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>37.25</v>
+        <v>20.25</v>
       </c>
       <c r="E46" s="10" t="n">
         <v>55</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E47" s="10" t="n">
         <v>70</v>
@@ -1629,19 +1629,19 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Varas C24 63 × 150 afastadas de 0,60</t>
+          <t>Asnas intermédias de linha alteada GL24h (vão 11,60 m)</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>184.6</v>
+        <v>1</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>8</v>
+        <v>632.5</v>
       </c>
       <c r="F48" s="11">
         <f>D48*E48</f>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Frechais 75 × 200 sobre o topo das paredes</t>
+          <t>Varas C24 63 × 150 afastadas de 0,60</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -1665,10 +1665,10 @@
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>15.2</v>
+        <v>184.6</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F49" s="11">
         <f>D49*E49</f>
@@ -1683,19 +1683,19 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Revestimento em telha cerâmica de encaixe + ripas, contra-ripas, membrana respirável</t>
+          <t>Frechais 75 × 200 sobre o topo das paredes</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>107.16</v>
+        <v>15.2</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="F50" s="11">
         <f>D50*E50</f>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Isolamento da esteira do desvão R ≥ 7 (lã mineral soprada)</t>
+          <t>Revestimento em telha cerâmica de encaixe + ripas, contra-ripas, membrana respirável</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>80.64</v>
+        <v>107.16</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F51" s="11">
         <f>D51*E51</f>
@@ -1737,19 +1737,19 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Caleiras de zinco meia-cana 33</t>
+          <t>Isolamento da esteira do desvão R ≥ 7 (lã mineral soprada)</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>15.2</v>
+        <v>80.64</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F52" s="11">
         <f>D52*E52</f>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Tubos de queda pluviais em zinco Ø80 + troço inferior em ferro fundido</t>
+          <t>Caleiras de zinco meia-cana 33</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -1773,10 +1773,10 @@
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>24.2</v>
+        <v>15.2</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F53" s="11">
         <f>D53*E53</f>
@@ -1784,43 +1784,43 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Tubos de queda pluviais em zinco Ø80 + troço inferior em ferro fundido</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" s="11">
+        <f>D54*E54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>05 — Instalações elétricas e ITED</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>L05</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Tomadas 16 A (embutidas, aparelhagem corrente)</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="n">
-        <v>31</v>
-      </c>
-      <c r="E55" s="10" t="n">
-        <v>38</v>
-      </c>
-      <c r="F55" s="11">
-        <f>D55*E55</f>
-        <v/>
-      </c>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Pontos de luz (caixa + casquilho)</t>
+          <t>Tomadas 16 A (embutidas, aparelhagem corrente)</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -1839,10 +1839,10 @@
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F56" s="11">
         <f>D56*E56</f>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Comandos (interruptores / comutadores de escada)</t>
+          <t>Pontos de luz (caixa + casquilho)</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -1866,10 +1866,10 @@
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="F57" s="11">
         <f>D57*E57</f>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Tomadas RJ45 (ITED)</t>
+          <t>Comandos (interruptores / comutadores de escada)</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -1893,10 +1893,10 @@
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="F58" s="11">
         <f>D58*E58</f>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Circuitos dedicados (placa, forno, máquinas de lavar e secar, AQS, bomba de calor, VMC, portão)</t>
+          <t>Tomadas RJ45 (ITED)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -1920,10 +1920,10 @@
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E59" s="10" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="F59" s="11">
         <f>D59*E59</f>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Circuitos de estores elétricos (por piso)</t>
+          <t>Circuitos dedicados (placa, forno, máquinas de lavar e secar, AQS, bomba de calor, VMC, portão)</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -1947,10 +1947,10 @@
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F60" s="11">
         <f>D60*E60</f>
@@ -1965,19 +1965,19 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Quadro elétrico de 3 filas equipado (4 diferenciais 40 A 30 mA + disjuntores)</t>
+          <t>Circuitos de estores elétricos (por piso)</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>850</v>
+        <v>70</v>
       </c>
       <c r="F61" s="11">
         <f>D61*E61</f>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Caixa de entrada + ATI (ITED)</t>
+          <t>Quadro elétrico de 3 filas equipado (4 diferenciais 40 A 30 mA + disjuntores)</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>350</v>
+        <v>850</v>
       </c>
       <c r="F62" s="11">
         <f>D62*E62</f>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Elétrodo de terra em anel nas fundações + ligações equipotenciais</t>
+          <t>Caixa de entrada + ATI (ITED)</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -2031,7 +2031,7 @@
         <v>1</v>
       </c>
       <c r="E63" s="10" t="n">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="F63" s="11">
         <f>D63*E63</f>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Ventilação mecânica higrorregulável (ventilador + bocas + condutas)</t>
+          <t>Elétrodo de terra em anel nas fundações + ligações equipotenciais</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -2058,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>650</v>
+        <v>280</v>
       </c>
       <c r="F64" s="11">
         <f>D64*E64</f>
@@ -2066,43 +2066,43 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Ventilação mecânica higrorregulável (ventilador + bocas + condutas)</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>vg</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="10" t="n">
+        <v>650</v>
+      </c>
+      <c r="F65" s="11">
+        <f>D65*E65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>06 — Águas e esgotos (DR 23/95)</t>
         </is>
       </c>
-      <c r="B65" s="7" t="n"/>
-      <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
-      <c r="E65" s="7" t="n"/>
-      <c r="F65" s="7" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t>L06</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>Lava-loiças (cozinha, lavandaria) — torneiras</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D66" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="10" t="n">
-        <v>260</v>
-      </c>
-      <c r="F66" s="11">
-        <f>D66*E66</f>
-        <v/>
-      </c>
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="7" t="n"/>
+      <c r="F66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Ponto de água e esgoto para máquina de lavar loiça</t>
+          <t>Lava-loiças (cozinha, lavandaria) — torneiras</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="E67" s="10" t="n">
-        <v>85</v>
+        <v>260</v>
       </c>
       <c r="F67" s="11">
         <f>D67*E67</f>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Ponto de água e esgoto para máquina de lavar roupa</t>
+          <t>Ponto de água e esgoto para máquina de lavar loiça</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Sanitas suspensas com estrutura de apoio</t>
+          <t>Ponto de água e esgoto para máquina de lavar roupa</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -2175,10 +2175,10 @@
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="10" t="n">
-        <v>380</v>
+        <v>85</v>
       </c>
       <c r="F69" s="11">
         <f>D69*E69</f>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Lavatório pequeno</t>
+          <t>Sanitas suspensas com estrutura de apoio</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -2202,10 +2202,10 @@
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>190</v>
+        <v>380</v>
       </c>
       <c r="F70" s="11">
         <f>D70*E70</f>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Lavatórios + móveis + misturadoras</t>
+          <t>Lavatório pequeno</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
@@ -2232,7 +2232,7 @@
         <v>1</v>
       </c>
       <c r="E71" s="10" t="n">
-        <v>300</v>
+        <v>190</v>
       </c>
       <c r="F71" s="11">
         <f>D71*E71</f>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Banheira acrílica 170 + misturadora</t>
+          <t>Lavatórios + móveis + misturadoras</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -2259,7 +2259,7 @@
         <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F72" s="11">
         <f>D72*E72</f>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Torneira de rega exterior anticongelante</t>
+          <t>Banheira acrílica 170 + misturadora</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -2286,7 +2286,7 @@
         <v>1</v>
       </c>
       <c r="E73" s="10" t="n">
-        <v>90</v>
+        <v>600</v>
       </c>
       <c r="F73" s="11">
         <f>D73*E73</f>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Bomba de calor para AQS 200 L + grupo de segurança</t>
+          <t>Torneira de rega exterior anticongelante</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
@@ -2313,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>1650</v>
+        <v>90</v>
       </c>
       <c r="F74" s="11">
         <f>D74*E74</f>
@@ -2328,19 +2328,19 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Coletores AF/AQS, redutor de pressão, filtro, válvula de retenção, válvulas</t>
+          <t>Bomba de calor para AQS 200 L + grupo de segurança</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D75" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E75" s="10" t="n">
-        <v>950</v>
+        <v>1650</v>
       </c>
       <c r="F75" s="11">
         <f>D75*E75</f>
@@ -2355,19 +2355,19 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Distribuição em multicamada com manga (AF + AQS)</t>
+          <t>Coletores AF/AQS, redutor de pressão, filtro, válvula de retenção, válvulas</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>vg</t>
         </is>
       </c>
       <c r="D76" s="9" t="n">
-        <v>108.2</v>
+        <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>5.5</v>
+        <v>950</v>
       </c>
       <c r="F76" s="11">
         <f>D76*E76</f>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Tubos de queda de águas residuais em PVC Ø100 + ventilação primária</t>
+          <t>Distribuição em multicamada com manga (AF + AQS)</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -2391,10 +2391,10 @@
         </is>
       </c>
       <c r="D77" s="9" t="n">
-        <v>19.4</v>
+        <v>111.2</v>
       </c>
       <c r="E77" s="10" t="n">
-        <v>22</v>
+        <v>5.5</v>
       </c>
       <c r="F77" s="11">
         <f>D77*E77</f>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Coletor Ø100 enterrado sob a laje térrea + ramais Ø32/40/100 dos aparelhos</t>
+          <t>Tubos de queda de águas residuais em PVC Ø100 + ventilação primária</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
@@ -2418,10 +2418,10 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>23.65</v>
+        <v>19.4</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F78" s="11">
         <f>D78*E78</f>
@@ -2436,153 +2436,180 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Ligação à rede no limite (sem taxas da entidade gestora)</t>
+          <t>Coletor Ø100 enterrado sob a laje térrea + ramais Ø32/40/100 dos aparelhos</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D79" s="9" t="n">
-        <v>1</v>
+        <v>23.04</v>
       </c>
       <c r="E79" s="10" t="n">
-        <v>600</v>
+        <v>26</v>
       </c>
       <c r="F79" s="11">
         <f>D79*E79</f>
         <v/>
       </c>
     </row>
-    <row r="80"/>
-    <row r="81">
-      <c r="B81" s="12" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Ligação à rede no limite (sem taxas da entidade gestora)</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>vg</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="F80" s="11">
+        <f>D80*E80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81"/>
+    <row r="82">
+      <c r="B82" s="12" t="inlineStr">
         <is>
           <t>RESUMO POR CAPÍTULO</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>01 — Estaleiro, estudos, movimento de terras</t>
-        </is>
-      </c>
-      <c r="F82" s="13">
-        <f>SUMIF($A$7:$A$79,"L01",$F$7:$F$79)</f>
-        <v/>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>02 — Fundações e laje térrea</t>
+          <t>01 — Estaleiro, estudos, movimento de terras</t>
         </is>
       </c>
       <c r="F83" s="13">
-        <f>SUMIF($A$7:$A$79,"L02",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L01",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>03 — Estrutura e alvenarias em elevação</t>
+          <t>02 — Fundações e laje térrea</t>
         </is>
       </c>
       <c r="F84" s="13">
-        <f>SUMIF($A$7:$A$79,"L03",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L02",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>04 — Estrutura da cobertura, revestimento, caleiras</t>
+          <t>03 — Estrutura e alvenarias em elevação</t>
         </is>
       </c>
       <c r="F85" s="13">
-        <f>SUMIF($A$7:$A$79,"L04",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L03",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>05 — Instalações elétricas e ITED</t>
+          <t>04 — Estrutura da cobertura, revestimento, caleiras</t>
         </is>
       </c>
       <c r="F86" s="13">
-        <f>SUMIF($A$7:$A$79,"L05",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L04",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>05 — Instalações elétricas e ITED</t>
+        </is>
+      </c>
+      <c r="F87" s="13">
+        <f>SUMIF($A$7:$A$80,"L05",$F$7:$F$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>06 — Águas e esgotos (DR 23/95)</t>
         </is>
       </c>
-      <c r="F87" s="13">
-        <f>SUMIF($A$7:$A$79,"L06",$F$7:$F$79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="12" t="inlineStr">
+      <c r="F88" s="13">
+        <f>SUMIF($A$7:$A$80,"L06",$F$7:$F$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="12" t="inlineStr">
         <is>
           <t>TOTAL s/ IVA</t>
         </is>
       </c>
-      <c r="F88" s="14">
-        <f>SUM(F7:F79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="2" t="inlineStr">
+      <c r="F89" s="14">
+        <f>SUM(F7:F80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>IVA</t>
         </is>
       </c>
-      <c r="F89" s="13">
-        <f>F88*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="12" t="inlineStr">
+      <c r="F90" s="13">
+        <f>F89*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="12" t="inlineStr">
         <is>
           <t>TOTAL c/ IVA</t>
         </is>
       </c>
-      <c r="F90" s="14">
-        <f>F88+F89</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="2" t="inlineStr">
+      <c r="F91" s="14">
+        <f>F89+F90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Rácio € s/ IVA / m² de área útil medida (135,60 m²)</t>
         </is>
       </c>
-      <c r="F91" s="15">
-        <f>F88/135.6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92"/>
-    <row r="93">
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>Excluídos : caixilharias exteriores, gessos e isolamento das paredes, betonilhas, revestimentos, pinturas, aquecimento (emissores + bomba de calor), arranjos exteriores, ramais das entidades gestoras.</t>
-        </is>
-      </c>
-    </row>
+      <c r="F92" s="15">
+        <f>F89/135.6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93"/>
     <row r="94">
       <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Excluídos : caixilharias exteriores, gessos e isolamento das paredes, betonilhas, revestimentos, pinturas, aquecimento (emissores + bomba de calor), arranjos exteriores, ramais das entidades gestoras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="3" t="inlineStr">
         <is>
           <t>Preços indicativos não contratuais : o ConstruPilot não garante os preços ; substituir pela base de preços da empresa antes de qualquer envio ao cliente.</t>
         </is>
@@ -4232,7 +4259,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Bomba de calor ar/água (hipótese de aquecimento) (Arrumos / zona técnica)</t>
+          <t>PAC air/eau (Arrumos / zona técnica)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -4587,7 +4614,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5.55</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="3">
@@ -4627,7 +4654,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -4667,7 +4694,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>4.25</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5">
@@ -4707,7 +4734,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="6">
@@ -4747,7 +4774,7 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="7">
@@ -4787,7 +4814,7 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.05</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="8">
@@ -4827,7 +4854,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="9">
@@ -4867,7 +4894,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.55</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Lote 5 PT: modo stand Web Summit, Assistente offline, nota sísmica de Lisboa, limpeza do francês nos PDF; SW v10
</commit_message>
<xml_diff>
--- a/frontend/public/demo-assets/Orcamento_Moradia_Martins.xlsx
+++ b/frontend/public/demo-assets/Orcamento_Moradia_Martins.xlsx
@@ -36,7 +36,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="000E4D4A"/>
+      <color rgb="00203B2D"/>
       <sz val="14"/>
     </font>
     <font>
@@ -74,12 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000E4D4A"/>
+        <fgColor rgb="00203B2D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7EDED"/>
+        <fgColor rgb="00E9EBEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Madres de lamelado colado GL24h 115 × 360 (×5)</t>
+          <t>Madres de lamelado colado GL24h 100 × 240 (×5)</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
@@ -1584,7 +1584,7 @@
         </is>
       </c>
       <c r="D46" s="9" t="n">
-        <v>37.25</v>
+        <v>20.25</v>
       </c>
       <c r="E46" s="10" t="n">
         <v>55</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D47" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E47" s="10" t="n">
         <v>70</v>
@@ -1629,19 +1629,19 @@
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Varas C24 63 × 150 afastadas de 0,60</t>
+          <t>Asnas intermédias de linha alteada GL24h (vão 11,60 m)</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D48" s="9" t="n">
-        <v>184.6</v>
+        <v>1</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>8</v>
+        <v>632.5</v>
       </c>
       <c r="F48" s="11">
         <f>D48*E48</f>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>Frechais 75 × 200 sobre o topo das paredes</t>
+          <t>Varas C24 63 × 150 afastadas de 0,60</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
@@ -1665,10 +1665,10 @@
         </is>
       </c>
       <c r="D49" s="9" t="n">
-        <v>15.2</v>
+        <v>184.6</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F49" s="11">
         <f>D49*E49</f>
@@ -1683,19 +1683,19 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Revestimento em telha cerâmica de encaixe + ripas, contra-ripas, membrana respirável</t>
+          <t>Frechais 75 × 200 sobre o topo das paredes</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D50" s="9" t="n">
-        <v>107.16</v>
+        <v>15.2</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="F50" s="11">
         <f>D50*E50</f>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>Isolamento da esteira do desvão R ≥ 7 (lã mineral soprada)</t>
+          <t>Revestimento em telha cerâmica de encaixe + ripas, contra-ripas, membrana respirável</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="D51" s="9" t="n">
-        <v>80.64</v>
+        <v>107.16</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="F51" s="11">
         <f>D51*E51</f>
@@ -1737,19 +1737,19 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Caleiras de zinco meia-cana 33</t>
+          <t>Isolamento da esteira do desvão R ≥ 7 (lã mineral soprada)</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D52" s="9" t="n">
-        <v>15.2</v>
+        <v>80.64</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F52" s="11">
         <f>D52*E52</f>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>Tubos de queda pluviais em zinco Ø80 + troço inferior em ferro fundido</t>
+          <t>Caleiras de zinco meia-cana 33</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -1773,10 +1773,10 @@
         </is>
       </c>
       <c r="D53" s="9" t="n">
-        <v>24.2</v>
+        <v>15.2</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F53" s="11">
         <f>D53*E53</f>
@@ -1784,43 +1784,43 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>L04</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>Tubos de queda pluviais em zinco Ø80 + troço inferior em ferro fundido</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F54" s="11">
+        <f>D54*E54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>05 — Instalações elétricas e ITED</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
-        <is>
-          <t>L05</t>
-        </is>
-      </c>
-      <c r="B55" s="8" t="inlineStr">
-        <is>
-          <t>Tomadas 16 A (embutidas, aparelhagem corrente)</t>
-        </is>
-      </c>
-      <c r="C55" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D55" s="9" t="n">
-        <v>31</v>
-      </c>
-      <c r="E55" s="10" t="n">
-        <v>38</v>
-      </c>
-      <c r="F55" s="11">
-        <f>D55*E55</f>
-        <v/>
-      </c>
+      <c r="B55" s="7" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="7" t="n"/>
+      <c r="E55" s="7" t="n"/>
+      <c r="F55" s="7" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>Pontos de luz (caixa + casquilho)</t>
+          <t>Tomadas 16 A (embutidas, aparelhagem corrente)</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -1839,10 +1839,10 @@
         </is>
       </c>
       <c r="D56" s="9" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F56" s="11">
         <f>D56*E56</f>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>Comandos (interruptores / comutadores de escada)</t>
+          <t>Pontos de luz (caixa + casquilho)</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -1866,10 +1866,10 @@
         </is>
       </c>
       <c r="D57" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="F57" s="11">
         <f>D57*E57</f>
@@ -1884,7 +1884,7 @@
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>Tomadas RJ45 (ITED)</t>
+          <t>Comandos (interruptores / comutadores de escada)</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -1893,10 +1893,10 @@
         </is>
       </c>
       <c r="D58" s="9" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="F58" s="11">
         <f>D58*E58</f>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>Circuitos dedicados (placa, forno, máquinas de lavar e secar, AQS, bomba de calor, VMC, portão)</t>
+          <t>Tomadas RJ45 (ITED)</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -1920,10 +1920,10 @@
         </is>
       </c>
       <c r="D59" s="9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E59" s="10" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="F59" s="11">
         <f>D59*E59</f>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>Circuitos de estores elétricos (por piso)</t>
+          <t>Circuitos dedicados (placa, forno, máquinas de lavar e secar, AQS, bomba de calor, VMC, portão)</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -1947,10 +1947,10 @@
         </is>
       </c>
       <c r="D60" s="9" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F60" s="11">
         <f>D60*E60</f>
@@ -1965,19 +1965,19 @@
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>Quadro elétrico de 3 filas equipado (4 diferenciais 40 A 30 mA + disjuntores)</t>
+          <t>Circuitos de estores elétricos (por piso)</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D61" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>850</v>
+        <v>70</v>
       </c>
       <c r="F61" s="11">
         <f>D61*E61</f>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>Caixa de entrada + ATI (ITED)</t>
+          <t>Quadro elétrico de 3 filas equipado (4 diferenciais 40 A 30 mA + disjuntores)</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -2004,7 +2004,7 @@
         <v>1</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>350</v>
+        <v>850</v>
       </c>
       <c r="F62" s="11">
         <f>D62*E62</f>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>Elétrodo de terra em anel nas fundações + ligações equipotenciais</t>
+          <t>Caixa de entrada + ATI (ITED)</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -2031,7 +2031,7 @@
         <v>1</v>
       </c>
       <c r="E63" s="10" t="n">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="F63" s="11">
         <f>D63*E63</f>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>Ventilação mecânica higrorregulável (ventilador + bocas + condutas)</t>
+          <t>Elétrodo de terra em anel nas fundações + ligações equipotenciais</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -2058,7 +2058,7 @@
         <v>1</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>650</v>
+        <v>280</v>
       </c>
       <c r="F64" s="11">
         <f>D64*E64</f>
@@ -2066,43 +2066,43 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>L05</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>Ventilação mecânica higrorregulável (ventilador + bocas + condutas)</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>vg</t>
+        </is>
+      </c>
+      <c r="D65" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="10" t="n">
+        <v>650</v>
+      </c>
+      <c r="F65" s="11">
+        <f>D65*E65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
         <is>
           <t>06 — Águas e esgotos (DR 23/95)</t>
         </is>
       </c>
-      <c r="B65" s="7" t="n"/>
-      <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
-      <c r="E65" s="7" t="n"/>
-      <c r="F65" s="7" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t>L06</t>
-        </is>
-      </c>
-      <c r="B66" s="8" t="inlineStr">
-        <is>
-          <t>Lava-loiças (cozinha, lavandaria) — torneiras</t>
-        </is>
-      </c>
-      <c r="C66" s="8" t="inlineStr">
-        <is>
-          <t>un</t>
-        </is>
-      </c>
-      <c r="D66" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="10" t="n">
-        <v>260</v>
-      </c>
-      <c r="F66" s="11">
-        <f>D66*E66</f>
-        <v/>
-      </c>
+      <c r="B66" s="7" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="7" t="n"/>
+      <c r="E66" s="7" t="n"/>
+      <c r="F66" s="7" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>Ponto de água e esgoto para máquina de lavar loiça</t>
+          <t>Lava-loiças (cozinha, lavandaria) — torneiras</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -2124,7 +2124,7 @@
         <v>1</v>
       </c>
       <c r="E67" s="10" t="n">
-        <v>85</v>
+        <v>260</v>
       </c>
       <c r="F67" s="11">
         <f>D67*E67</f>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>Ponto de água e esgoto para máquina de lavar roupa</t>
+          <t>Ponto de água e esgoto para máquina de lavar loiça</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Sanitas suspensas com estrutura de apoio</t>
+          <t>Ponto de água e esgoto para máquina de lavar roupa</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -2175,10 +2175,10 @@
         </is>
       </c>
       <c r="D69" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="10" t="n">
-        <v>380</v>
+        <v>85</v>
       </c>
       <c r="F69" s="11">
         <f>D69*E69</f>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>Lavatório pequeno</t>
+          <t>Sanitas suspensas com estrutura de apoio</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
@@ -2202,10 +2202,10 @@
         </is>
       </c>
       <c r="D70" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>190</v>
+        <v>380</v>
       </c>
       <c r="F70" s="11">
         <f>D70*E70</f>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>Lavatórios + móveis + misturadoras</t>
+          <t>Lavatório pequeno</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
@@ -2232,7 +2232,7 @@
         <v>1</v>
       </c>
       <c r="E71" s="10" t="n">
-        <v>300</v>
+        <v>190</v>
       </c>
       <c r="F71" s="11">
         <f>D71*E71</f>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Banheira acrílica 170 + misturadora</t>
+          <t>Lavatórios + móveis + misturadoras</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
@@ -2259,7 +2259,7 @@
         <v>1</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F72" s="11">
         <f>D72*E72</f>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>Torneira de rega exterior anticongelante</t>
+          <t>Banheira acrílica 170 + misturadora</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -2286,7 +2286,7 @@
         <v>1</v>
       </c>
       <c r="E73" s="10" t="n">
-        <v>90</v>
+        <v>600</v>
       </c>
       <c r="F73" s="11">
         <f>D73*E73</f>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>Bomba de calor para AQS 200 L + grupo de segurança</t>
+          <t>Torneira de rega exterior anticongelante</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
@@ -2313,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>1650</v>
+        <v>90</v>
       </c>
       <c r="F74" s="11">
         <f>D74*E74</f>
@@ -2328,19 +2328,19 @@
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>Coletores AF/AQS, redutor de pressão, filtro, válvula de retenção, válvulas</t>
+          <t>Bomba de calor para AQS 200 L + grupo de segurança</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>un</t>
         </is>
       </c>
       <c r="D75" s="9" t="n">
         <v>1</v>
       </c>
       <c r="E75" s="10" t="n">
-        <v>950</v>
+        <v>1650</v>
       </c>
       <c r="F75" s="11">
         <f>D75*E75</f>
@@ -2355,19 +2355,19 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>Distribuição em multicamada com manga (AF + AQS)</t>
+          <t>Coletores AF/AQS, redutor de pressão, filtro, válvula de retenção, válvulas</t>
         </is>
       </c>
       <c r="C76" s="8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>vg</t>
         </is>
       </c>
       <c r="D76" s="9" t="n">
-        <v>108.2</v>
+        <v>1</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>5.5</v>
+        <v>950</v>
       </c>
       <c r="F76" s="11">
         <f>D76*E76</f>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>Tubos de queda de águas residuais em PVC Ø100 + ventilação primária</t>
+          <t>Distribuição em multicamada com manga (AF + AQS)</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -2391,10 +2391,10 @@
         </is>
       </c>
       <c r="D77" s="9" t="n">
-        <v>19.4</v>
+        <v>111.2</v>
       </c>
       <c r="E77" s="10" t="n">
-        <v>22</v>
+        <v>5.5</v>
       </c>
       <c r="F77" s="11">
         <f>D77*E77</f>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>Coletor Ø100 enterrado sob a laje térrea + ramais Ø32/40/100 dos aparelhos</t>
+          <t>Tubos de queda de águas residuais em PVC Ø100 + ventilação primária</t>
         </is>
       </c>
       <c r="C78" s="8" t="inlineStr">
@@ -2418,10 +2418,10 @@
         </is>
       </c>
       <c r="D78" s="9" t="n">
-        <v>23.65</v>
+        <v>19.4</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F78" s="11">
         <f>D78*E78</f>
@@ -2436,153 +2436,180 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Ligação à rede no limite (sem taxas da entidade gestora)</t>
+          <t>Coletor Ø100 enterrado sob a laje térrea + ramais Ø32/40/100 dos aparelhos</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>vg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D79" s="9" t="n">
-        <v>1</v>
+        <v>23.04</v>
       </c>
       <c r="E79" s="10" t="n">
-        <v>600</v>
+        <v>26</v>
       </c>
       <c r="F79" s="11">
         <f>D79*E79</f>
         <v/>
       </c>
     </row>
-    <row r="80"/>
-    <row r="81">
-      <c r="B81" s="12" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>L06</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>Ligação à rede no limite (sem taxas da entidade gestora)</t>
+        </is>
+      </c>
+      <c r="C80" s="8" t="inlineStr">
+        <is>
+          <t>vg</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="10" t="n">
+        <v>600</v>
+      </c>
+      <c r="F80" s="11">
+        <f>D80*E80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81"/>
+    <row r="82">
+      <c r="B82" s="12" t="inlineStr">
         <is>
           <t>RESUMO POR CAPÍTULO</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>01 — Estaleiro, estudos, movimento de terras</t>
-        </is>
-      </c>
-      <c r="F82" s="13">
-        <f>SUMIF($A$7:$A$79,"L01",$F$7:$F$79)</f>
-        <v/>
       </c>
     </row>
     <row r="83">
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>02 — Fundações e laje térrea</t>
+          <t>01 — Estaleiro, estudos, movimento de terras</t>
         </is>
       </c>
       <c r="F83" s="13">
-        <f>SUMIF($A$7:$A$79,"L02",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L01",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>03 — Estrutura e alvenarias em elevação</t>
+          <t>02 — Fundações e laje térrea</t>
         </is>
       </c>
       <c r="F84" s="13">
-        <f>SUMIF($A$7:$A$79,"L03",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L02",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>04 — Estrutura da cobertura, revestimento, caleiras</t>
+          <t>03 — Estrutura e alvenarias em elevação</t>
         </is>
       </c>
       <c r="F85" s="13">
-        <f>SUMIF($A$7:$A$79,"L04",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L03",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>05 — Instalações elétricas e ITED</t>
+          <t>04 — Estrutura da cobertura, revestimento, caleiras</t>
         </is>
       </c>
       <c r="F86" s="13">
-        <f>SUMIF($A$7:$A$79,"L05",$F$7:$F$79)</f>
+        <f>SUMIF($A$7:$A$80,"L04",$F$7:$F$80)</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>05 — Instalações elétricas e ITED</t>
+        </is>
+      </c>
+      <c r="F87" s="13">
+        <f>SUMIF($A$7:$A$80,"L05",$F$7:$F$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>06 — Águas e esgotos (DR 23/95)</t>
         </is>
       </c>
-      <c r="F87" s="13">
-        <f>SUMIF($A$7:$A$79,"L06",$F$7:$F$79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="B88" s="12" t="inlineStr">
+      <c r="F88" s="13">
+        <f>SUMIF($A$7:$A$80,"L06",$F$7:$F$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="12" t="inlineStr">
         <is>
           <t>TOTAL s/ IVA</t>
         </is>
       </c>
-      <c r="F88" s="14">
-        <f>SUM(F7:F79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="B89" s="2" t="inlineStr">
+      <c r="F89" s="14">
+        <f>SUM(F7:F80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>IVA</t>
         </is>
       </c>
-      <c r="F89" s="13">
-        <f>F88*$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="12" t="inlineStr">
+      <c r="F90" s="13">
+        <f>F89*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="12" t="inlineStr">
         <is>
           <t>TOTAL c/ IVA</t>
         </is>
       </c>
-      <c r="F90" s="14">
-        <f>F88+F89</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="2" t="inlineStr">
+      <c r="F91" s="14">
+        <f>F89+F90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Rácio € s/ IVA / m² de área útil medida (135,60 m²)</t>
         </is>
       </c>
-      <c r="F91" s="15">
-        <f>F88/135.6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92"/>
-    <row r="93">
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>Excluídos : caixilharias exteriores, gessos e isolamento das paredes, betonilhas, revestimentos, pinturas, aquecimento (emissores + bomba de calor), arranjos exteriores, ramais das entidades gestoras.</t>
-        </is>
-      </c>
-    </row>
+      <c r="F92" s="15">
+        <f>F89/135.6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93"/>
     <row r="94">
       <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Excluídos : caixilharias exteriores, gessos e isolamento das paredes, betonilhas, revestimentos, pinturas, aquecimento (emissores + bomba de calor), arranjos exteriores, ramais das entidades gestoras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="B95" s="3" t="inlineStr">
         <is>
           <t>Preços indicativos não contratuais : o ConstruPilot não garante os preços ; substituir pela base de preços da empresa antes de qualquer envio ao cliente.</t>
         </is>
@@ -4232,7 +4259,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Bomba de calor ar/água (hipótese de aquecimento) (Arrumos / zona técnica)</t>
+          <t>PAC air/eau (Arrumos / zona técnica)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -4587,7 +4614,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5.55</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="3">
@@ -4627,7 +4654,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4.9</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -4667,7 +4694,7 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>4.25</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="5">
@@ -4707,7 +4734,7 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.25</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="6">
@@ -4747,7 +4774,7 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.7</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="7">
@@ -4787,7 +4814,7 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>1.05</v>
+        <v>1.12</v>
       </c>
     </row>
     <row r="8">
@@ -4827,7 +4854,7 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="9">
@@ -4867,7 +4894,7 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>0.55</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="10">

</xml_diff>